<commit_message>
Add separate FF stock batch tracking
</commit_message>
<xml_diff>
--- a/public/ff-stock-import-template.xlsx
+++ b/public/ff-stock-import-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Остатки ФФ" sheetId="1" r:id="R65c8e480a4004033"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Остатки ФФ" sheetId="1" r:id="R7ae5f3bf5ec24dd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -504,8 +504,9 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -514,529 +515,634 @@
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Заполните строки ниже. Срок годности необязателен; используйте формат ДД.ММ.ГГГГ.</x:v>
+        <x:v>Каждая строка — отдельная партия. Номер партии и срок годности необязательны; срок укажите в формате ДД.ММ.ГГГГ.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
+      <x:c r="D2" s="8"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="17" t="str">
         <x:v>Артикул</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
+        <x:v>Партия</x:v>
+      </x:c>
+      <x:c r="C4" s="18" t="str">
         <x:v>Количество</x:v>
       </x:c>
-      <x:c r="C4" s="19" t="str">
+      <x:c r="D4" s="19" t="str">
         <x:v>Срок годности</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="39"/>
-      <x:c r="B5" s="42"/>
-      <x:c r="C5" s="45"/>
+      <x:c r="B5" s="31"/>
+      <x:c r="C5" s="42"/>
+      <x:c r="D5" s="45"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="40"/>
-      <x:c r="B6" s="43"/>
-      <x:c r="C6" s="46"/>
+      <x:c r="B6" s="34"/>
+      <x:c r="C6" s="43"/>
+      <x:c r="D6" s="46"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="40"/>
-      <x:c r="B7" s="43"/>
-      <x:c r="C7" s="46"/>
+      <x:c r="B7" s="34"/>
+      <x:c r="C7" s="43"/>
+      <x:c r="D7" s="46"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="40"/>
-      <x:c r="B8" s="43"/>
-      <x:c r="C8" s="46"/>
+      <x:c r="B8" s="34"/>
+      <x:c r="C8" s="43"/>
+      <x:c r="D8" s="46"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="40"/>
-      <x:c r="B9" s="43"/>
-      <x:c r="C9" s="46"/>
+      <x:c r="B9" s="34"/>
+      <x:c r="C9" s="43"/>
+      <x:c r="D9" s="46"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="40"/>
-      <x:c r="B10" s="43"/>
-      <x:c r="C10" s="46"/>
+      <x:c r="B10" s="34"/>
+      <x:c r="C10" s="43"/>
+      <x:c r="D10" s="46"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="40"/>
-      <x:c r="B11" s="43"/>
-      <x:c r="C11" s="46"/>
+      <x:c r="B11" s="34"/>
+      <x:c r="C11" s="43"/>
+      <x:c r="D11" s="46"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40"/>
-      <x:c r="B12" s="43"/>
-      <x:c r="C12" s="46"/>
+      <x:c r="B12" s="34"/>
+      <x:c r="C12" s="43"/>
+      <x:c r="D12" s="46"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="40"/>
-      <x:c r="B13" s="43"/>
-      <x:c r="C13" s="46"/>
+      <x:c r="B13" s="34"/>
+      <x:c r="C13" s="43"/>
+      <x:c r="D13" s="46"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40"/>
-      <x:c r="B14" s="43"/>
-      <x:c r="C14" s="46"/>
+      <x:c r="B14" s="34"/>
+      <x:c r="C14" s="43"/>
+      <x:c r="D14" s="46"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40"/>
-      <x:c r="B15" s="43"/>
-      <x:c r="C15" s="46"/>
+      <x:c r="B15" s="34"/>
+      <x:c r="C15" s="43"/>
+      <x:c r="D15" s="46"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="40"/>
-      <x:c r="B16" s="43"/>
-      <x:c r="C16" s="46"/>
+      <x:c r="B16" s="34"/>
+      <x:c r="C16" s="43"/>
+      <x:c r="D16" s="46"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40"/>
-      <x:c r="B17" s="43"/>
-      <x:c r="C17" s="46"/>
+      <x:c r="B17" s="34"/>
+      <x:c r="C17" s="43"/>
+      <x:c r="D17" s="46"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40"/>
-      <x:c r="B18" s="43"/>
-      <x:c r="C18" s="46"/>
+      <x:c r="B18" s="34"/>
+      <x:c r="C18" s="43"/>
+      <x:c r="D18" s="46"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="40"/>
-      <x:c r="B19" s="43"/>
-      <x:c r="C19" s="46"/>
+      <x:c r="B19" s="34"/>
+      <x:c r="C19" s="43"/>
+      <x:c r="D19" s="46"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="40"/>
-      <x:c r="B20" s="43"/>
-      <x:c r="C20" s="46"/>
+      <x:c r="B20" s="34"/>
+      <x:c r="C20" s="43"/>
+      <x:c r="D20" s="46"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="40"/>
-      <x:c r="B21" s="43"/>
-      <x:c r="C21" s="46"/>
+      <x:c r="B21" s="34"/>
+      <x:c r="C21" s="43"/>
+      <x:c r="D21" s="46"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="40"/>
-      <x:c r="B22" s="43"/>
-      <x:c r="C22" s="46"/>
+      <x:c r="B22" s="34"/>
+      <x:c r="C22" s="43"/>
+      <x:c r="D22" s="46"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="40"/>
-      <x:c r="B23" s="43"/>
-      <x:c r="C23" s="46"/>
+      <x:c r="B23" s="34"/>
+      <x:c r="C23" s="43"/>
+      <x:c r="D23" s="46"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="40"/>
-      <x:c r="B24" s="43"/>
-      <x:c r="C24" s="46"/>
+      <x:c r="B24" s="34"/>
+      <x:c r="C24" s="43"/>
+      <x:c r="D24" s="46"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="40"/>
-      <x:c r="B25" s="43"/>
-      <x:c r="C25" s="46"/>
+      <x:c r="B25" s="34"/>
+      <x:c r="C25" s="43"/>
+      <x:c r="D25" s="46"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="40"/>
-      <x:c r="B26" s="43"/>
-      <x:c r="C26" s="46"/>
+      <x:c r="B26" s="34"/>
+      <x:c r="C26" s="43"/>
+      <x:c r="D26" s="46"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="40"/>
-      <x:c r="B27" s="43"/>
-      <x:c r="C27" s="46"/>
+      <x:c r="B27" s="34"/>
+      <x:c r="C27" s="43"/>
+      <x:c r="D27" s="46"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="40"/>
-      <x:c r="B28" s="43"/>
-      <x:c r="C28" s="46"/>
+      <x:c r="B28" s="34"/>
+      <x:c r="C28" s="43"/>
+      <x:c r="D28" s="46"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="40"/>
-      <x:c r="B29" s="43"/>
-      <x:c r="C29" s="46"/>
+      <x:c r="B29" s="34"/>
+      <x:c r="C29" s="43"/>
+      <x:c r="D29" s="46"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="40"/>
-      <x:c r="B30" s="43"/>
-      <x:c r="C30" s="46"/>
+      <x:c r="B30" s="34"/>
+      <x:c r="C30" s="43"/>
+      <x:c r="D30" s="46"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="40"/>
-      <x:c r="B31" s="43"/>
-      <x:c r="C31" s="46"/>
+      <x:c r="B31" s="34"/>
+      <x:c r="C31" s="43"/>
+      <x:c r="D31" s="46"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="40"/>
-      <x:c r="B32" s="43"/>
-      <x:c r="C32" s="46"/>
+      <x:c r="B32" s="34"/>
+      <x:c r="C32" s="43"/>
+      <x:c r="D32" s="46"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="40"/>
-      <x:c r="B33" s="43"/>
-      <x:c r="C33" s="46"/>
+      <x:c r="B33" s="34"/>
+      <x:c r="C33" s="43"/>
+      <x:c r="D33" s="46"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="40"/>
-      <x:c r="B34" s="43"/>
-      <x:c r="C34" s="46"/>
+      <x:c r="B34" s="34"/>
+      <x:c r="C34" s="43"/>
+      <x:c r="D34" s="46"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="40"/>
-      <x:c r="B35" s="43"/>
-      <x:c r="C35" s="46"/>
+      <x:c r="B35" s="34"/>
+      <x:c r="C35" s="43"/>
+      <x:c r="D35" s="46"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="40"/>
-      <x:c r="B36" s="43"/>
-      <x:c r="C36" s="46"/>
+      <x:c r="B36" s="34"/>
+      <x:c r="C36" s="43"/>
+      <x:c r="D36" s="46"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="40"/>
-      <x:c r="B37" s="43"/>
-      <x:c r="C37" s="46"/>
+      <x:c r="B37" s="34"/>
+      <x:c r="C37" s="43"/>
+      <x:c r="D37" s="46"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="40"/>
-      <x:c r="B38" s="43"/>
-      <x:c r="C38" s="46"/>
+      <x:c r="B38" s="34"/>
+      <x:c r="C38" s="43"/>
+      <x:c r="D38" s="46"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="40"/>
-      <x:c r="B39" s="43"/>
-      <x:c r="C39" s="46"/>
+      <x:c r="B39" s="34"/>
+      <x:c r="C39" s="43"/>
+      <x:c r="D39" s="46"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="40"/>
-      <x:c r="B40" s="43"/>
-      <x:c r="C40" s="46"/>
+      <x:c r="B40" s="34"/>
+      <x:c r="C40" s="43"/>
+      <x:c r="D40" s="46"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="40"/>
-      <x:c r="B41" s="43"/>
-      <x:c r="C41" s="46"/>
+      <x:c r="B41" s="34"/>
+      <x:c r="C41" s="43"/>
+      <x:c r="D41" s="46"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="40"/>
-      <x:c r="B42" s="43"/>
-      <x:c r="C42" s="46"/>
+      <x:c r="B42" s="34"/>
+      <x:c r="C42" s="43"/>
+      <x:c r="D42" s="46"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="40"/>
-      <x:c r="B43" s="43"/>
-      <x:c r="C43" s="46"/>
+      <x:c r="B43" s="34"/>
+      <x:c r="C43" s="43"/>
+      <x:c r="D43" s="46"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="40"/>
-      <x:c r="B44" s="43"/>
-      <x:c r="C44" s="46"/>
+      <x:c r="B44" s="34"/>
+      <x:c r="C44" s="43"/>
+      <x:c r="D44" s="46"/>
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="40"/>
-      <x:c r="B45" s="43"/>
-      <x:c r="C45" s="46"/>
+      <x:c r="B45" s="34"/>
+      <x:c r="C45" s="43"/>
+      <x:c r="D45" s="46"/>
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="40"/>
-      <x:c r="B46" s="43"/>
-      <x:c r="C46" s="46"/>
+      <x:c r="B46" s="34"/>
+      <x:c r="C46" s="43"/>
+      <x:c r="D46" s="46"/>
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="40"/>
-      <x:c r="B47" s="43"/>
-      <x:c r="C47" s="46"/>
+      <x:c r="B47" s="34"/>
+      <x:c r="C47" s="43"/>
+      <x:c r="D47" s="46"/>
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="40"/>
-      <x:c r="B48" s="43"/>
-      <x:c r="C48" s="46"/>
+      <x:c r="B48" s="34"/>
+      <x:c r="C48" s="43"/>
+      <x:c r="D48" s="46"/>
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="40"/>
-      <x:c r="B49" s="43"/>
-      <x:c r="C49" s="46"/>
+      <x:c r="B49" s="34"/>
+      <x:c r="C49" s="43"/>
+      <x:c r="D49" s="46"/>
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="40"/>
-      <x:c r="B50" s="43"/>
-      <x:c r="C50" s="46"/>
+      <x:c r="B50" s="34"/>
+      <x:c r="C50" s="43"/>
+      <x:c r="D50" s="46"/>
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="40"/>
-      <x:c r="B51" s="43"/>
-      <x:c r="C51" s="46"/>
+      <x:c r="B51" s="34"/>
+      <x:c r="C51" s="43"/>
+      <x:c r="D51" s="46"/>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="40"/>
-      <x:c r="B52" s="43"/>
-      <x:c r="C52" s="46"/>
+      <x:c r="B52" s="34"/>
+      <x:c r="C52" s="43"/>
+      <x:c r="D52" s="46"/>
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="40"/>
-      <x:c r="B53" s="43"/>
-      <x:c r="C53" s="46"/>
+      <x:c r="B53" s="34"/>
+      <x:c r="C53" s="43"/>
+      <x:c r="D53" s="46"/>
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="40"/>
-      <x:c r="B54" s="43"/>
-      <x:c r="C54" s="46"/>
+      <x:c r="B54" s="34"/>
+      <x:c r="C54" s="43"/>
+      <x:c r="D54" s="46"/>
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="40"/>
-      <x:c r="B55" s="43"/>
-      <x:c r="C55" s="46"/>
+      <x:c r="B55" s="34"/>
+      <x:c r="C55" s="43"/>
+      <x:c r="D55" s="46"/>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="40"/>
-      <x:c r="B56" s="43"/>
-      <x:c r="C56" s="46"/>
+      <x:c r="B56" s="34"/>
+      <x:c r="C56" s="43"/>
+      <x:c r="D56" s="46"/>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="40"/>
-      <x:c r="B57" s="43"/>
-      <x:c r="C57" s="46"/>
+      <x:c r="B57" s="34"/>
+      <x:c r="C57" s="43"/>
+      <x:c r="D57" s="46"/>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="40"/>
-      <x:c r="B58" s="43"/>
-      <x:c r="C58" s="46"/>
+      <x:c r="B58" s="34"/>
+      <x:c r="C58" s="43"/>
+      <x:c r="D58" s="46"/>
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="40"/>
-      <x:c r="B59" s="43"/>
-      <x:c r="C59" s="46"/>
+      <x:c r="B59" s="34"/>
+      <x:c r="C59" s="43"/>
+      <x:c r="D59" s="46"/>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="40"/>
-      <x:c r="B60" s="43"/>
-      <x:c r="C60" s="46"/>
+      <x:c r="B60" s="34"/>
+      <x:c r="C60" s="43"/>
+      <x:c r="D60" s="46"/>
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="40"/>
-      <x:c r="B61" s="43"/>
-      <x:c r="C61" s="46"/>
+      <x:c r="B61" s="34"/>
+      <x:c r="C61" s="43"/>
+      <x:c r="D61" s="46"/>
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="40"/>
-      <x:c r="B62" s="43"/>
-      <x:c r="C62" s="46"/>
+      <x:c r="B62" s="34"/>
+      <x:c r="C62" s="43"/>
+      <x:c r="D62" s="46"/>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="40"/>
-      <x:c r="B63" s="43"/>
-      <x:c r="C63" s="46"/>
+      <x:c r="B63" s="34"/>
+      <x:c r="C63" s="43"/>
+      <x:c r="D63" s="46"/>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="40"/>
-      <x:c r="B64" s="43"/>
-      <x:c r="C64" s="46"/>
+      <x:c r="B64" s="34"/>
+      <x:c r="C64" s="43"/>
+      <x:c r="D64" s="46"/>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="40"/>
-      <x:c r="B65" s="43"/>
-      <x:c r="C65" s="46"/>
+      <x:c r="B65" s="34"/>
+      <x:c r="C65" s="43"/>
+      <x:c r="D65" s="46"/>
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="40"/>
-      <x:c r="B66" s="43"/>
-      <x:c r="C66" s="46"/>
+      <x:c r="B66" s="34"/>
+      <x:c r="C66" s="43"/>
+      <x:c r="D66" s="46"/>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="40"/>
-      <x:c r="B67" s="43"/>
-      <x:c r="C67" s="46"/>
+      <x:c r="B67" s="34"/>
+      <x:c r="C67" s="43"/>
+      <x:c r="D67" s="46"/>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="40"/>
-      <x:c r="B68" s="43"/>
-      <x:c r="C68" s="46"/>
+      <x:c r="B68" s="34"/>
+      <x:c r="C68" s="43"/>
+      <x:c r="D68" s="46"/>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="40"/>
-      <x:c r="B69" s="43"/>
-      <x:c r="C69" s="46"/>
+      <x:c r="B69" s="34"/>
+      <x:c r="C69" s="43"/>
+      <x:c r="D69" s="46"/>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="40"/>
-      <x:c r="B70" s="43"/>
-      <x:c r="C70" s="46"/>
+      <x:c r="B70" s="34"/>
+      <x:c r="C70" s="43"/>
+      <x:c r="D70" s="46"/>
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="40"/>
-      <x:c r="B71" s="43"/>
-      <x:c r="C71" s="46"/>
+      <x:c r="B71" s="34"/>
+      <x:c r="C71" s="43"/>
+      <x:c r="D71" s="46"/>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="40"/>
-      <x:c r="B72" s="43"/>
-      <x:c r="C72" s="46"/>
+      <x:c r="B72" s="34"/>
+      <x:c r="C72" s="43"/>
+      <x:c r="D72" s="46"/>
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="40"/>
-      <x:c r="B73" s="43"/>
-      <x:c r="C73" s="46"/>
+      <x:c r="B73" s="34"/>
+      <x:c r="C73" s="43"/>
+      <x:c r="D73" s="46"/>
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="40"/>
-      <x:c r="B74" s="43"/>
-      <x:c r="C74" s="46"/>
+      <x:c r="B74" s="34"/>
+      <x:c r="C74" s="43"/>
+      <x:c r="D74" s="46"/>
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="40"/>
-      <x:c r="B75" s="43"/>
-      <x:c r="C75" s="46"/>
+      <x:c r="B75" s="34"/>
+      <x:c r="C75" s="43"/>
+      <x:c r="D75" s="46"/>
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="40"/>
-      <x:c r="B76" s="43"/>
-      <x:c r="C76" s="46"/>
+      <x:c r="B76" s="34"/>
+      <x:c r="C76" s="43"/>
+      <x:c r="D76" s="46"/>
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="40"/>
-      <x:c r="B77" s="43"/>
-      <x:c r="C77" s="46"/>
+      <x:c r="B77" s="34"/>
+      <x:c r="C77" s="43"/>
+      <x:c r="D77" s="46"/>
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="40"/>
-      <x:c r="B78" s="43"/>
-      <x:c r="C78" s="46"/>
+      <x:c r="B78" s="34"/>
+      <x:c r="C78" s="43"/>
+      <x:c r="D78" s="46"/>
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="40"/>
-      <x:c r="B79" s="43"/>
-      <x:c r="C79" s="46"/>
+      <x:c r="B79" s="34"/>
+      <x:c r="C79" s="43"/>
+      <x:c r="D79" s="46"/>
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="40"/>
-      <x:c r="B80" s="43"/>
-      <x:c r="C80" s="46"/>
+      <x:c r="B80" s="34"/>
+      <x:c r="C80" s="43"/>
+      <x:c r="D80" s="46"/>
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="40"/>
-      <x:c r="B81" s="43"/>
-      <x:c r="C81" s="46"/>
+      <x:c r="B81" s="34"/>
+      <x:c r="C81" s="43"/>
+      <x:c r="D81" s="46"/>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="40"/>
-      <x:c r="B82" s="43"/>
-      <x:c r="C82" s="46"/>
+      <x:c r="B82" s="34"/>
+      <x:c r="C82" s="43"/>
+      <x:c r="D82" s="46"/>
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="40"/>
-      <x:c r="B83" s="43"/>
-      <x:c r="C83" s="46"/>
+      <x:c r="B83" s="34"/>
+      <x:c r="C83" s="43"/>
+      <x:c r="D83" s="46"/>
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="40"/>
-      <x:c r="B84" s="43"/>
-      <x:c r="C84" s="46"/>
+      <x:c r="B84" s="34"/>
+      <x:c r="C84" s="43"/>
+      <x:c r="D84" s="46"/>
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="40"/>
-      <x:c r="B85" s="43"/>
-      <x:c r="C85" s="46"/>
+      <x:c r="B85" s="34"/>
+      <x:c r="C85" s="43"/>
+      <x:c r="D85" s="46"/>
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="40"/>
-      <x:c r="B86" s="43"/>
-      <x:c r="C86" s="46"/>
+      <x:c r="B86" s="34"/>
+      <x:c r="C86" s="43"/>
+      <x:c r="D86" s="46"/>
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="40"/>
-      <x:c r="B87" s="43"/>
-      <x:c r="C87" s="46"/>
+      <x:c r="B87" s="34"/>
+      <x:c r="C87" s="43"/>
+      <x:c r="D87" s="46"/>
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="40"/>
-      <x:c r="B88" s="43"/>
-      <x:c r="C88" s="46"/>
+      <x:c r="B88" s="34"/>
+      <x:c r="C88" s="43"/>
+      <x:c r="D88" s="46"/>
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="40"/>
-      <x:c r="B89" s="43"/>
-      <x:c r="C89" s="46"/>
+      <x:c r="B89" s="34"/>
+      <x:c r="C89" s="43"/>
+      <x:c r="D89" s="46"/>
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="40"/>
-      <x:c r="B90" s="43"/>
-      <x:c r="C90" s="46"/>
+      <x:c r="B90" s="34"/>
+      <x:c r="C90" s="43"/>
+      <x:c r="D90" s="46"/>
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="40"/>
-      <x:c r="B91" s="43"/>
-      <x:c r="C91" s="46"/>
+      <x:c r="B91" s="34"/>
+      <x:c r="C91" s="43"/>
+      <x:c r="D91" s="46"/>
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="40"/>
-      <x:c r="B92" s="43"/>
-      <x:c r="C92" s="46"/>
+      <x:c r="B92" s="34"/>
+      <x:c r="C92" s="43"/>
+      <x:c r="D92" s="46"/>
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="40"/>
-      <x:c r="B93" s="43"/>
-      <x:c r="C93" s="46"/>
+      <x:c r="B93" s="34"/>
+      <x:c r="C93" s="43"/>
+      <x:c r="D93" s="46"/>
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="40"/>
-      <x:c r="B94" s="43"/>
-      <x:c r="C94" s="46"/>
+      <x:c r="B94" s="34"/>
+      <x:c r="C94" s="43"/>
+      <x:c r="D94" s="46"/>
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="40"/>
-      <x:c r="B95" s="43"/>
-      <x:c r="C95" s="46"/>
+      <x:c r="B95" s="34"/>
+      <x:c r="C95" s="43"/>
+      <x:c r="D95" s="46"/>
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="40"/>
-      <x:c r="B96" s="43"/>
-      <x:c r="C96" s="46"/>
+      <x:c r="B96" s="34"/>
+      <x:c r="C96" s="43"/>
+      <x:c r="D96" s="46"/>
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="40"/>
-      <x:c r="B97" s="43"/>
-      <x:c r="C97" s="46"/>
+      <x:c r="B97" s="34"/>
+      <x:c r="C97" s="43"/>
+      <x:c r="D97" s="46"/>
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="40"/>
-      <x:c r="B98" s="43"/>
-      <x:c r="C98" s="46"/>
+      <x:c r="B98" s="34"/>
+      <x:c r="C98" s="43"/>
+      <x:c r="D98" s="46"/>
     </x:row>
     <x:row r="99">
       <x:c r="A99" s="40"/>
-      <x:c r="B99" s="43"/>
-      <x:c r="C99" s="46"/>
+      <x:c r="B99" s="34"/>
+      <x:c r="C99" s="43"/>
+      <x:c r="D99" s="46"/>
     </x:row>
     <x:row r="100">
       <x:c r="A100" s="40"/>
-      <x:c r="B100" s="43"/>
-      <x:c r="C100" s="46"/>
+      <x:c r="B100" s="34"/>
+      <x:c r="C100" s="43"/>
+      <x:c r="D100" s="46"/>
     </x:row>
     <x:row r="101">
       <x:c r="A101" s="40"/>
-      <x:c r="B101" s="43"/>
-      <x:c r="C101" s="46"/>
+      <x:c r="B101" s="34"/>
+      <x:c r="C101" s="43"/>
+      <x:c r="D101" s="46"/>
     </x:row>
     <x:row r="102">
       <x:c r="A102" s="40"/>
-      <x:c r="B102" s="43"/>
-      <x:c r="C102" s="46"/>
+      <x:c r="B102" s="34"/>
+      <x:c r="C102" s="43"/>
+      <x:c r="D102" s="46"/>
     </x:row>
     <x:row r="103">
       <x:c r="A103" s="40"/>
-      <x:c r="B103" s="43"/>
-      <x:c r="C103" s="46"/>
+      <x:c r="B103" s="34"/>
+      <x:c r="C103" s="43"/>
+      <x:c r="D103" s="46"/>
     </x:row>
     <x:row r="104">
       <x:c r="A104" s="41"/>
-      <x:c r="B104" s="44"/>
-      <x:c r="C104" s="47"/>
+      <x:c r="B104" s="37"/>
+      <x:c r="C104" s="44"/>
+      <x:c r="D104" s="47"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:C1"/>
-    <x:mergeCell ref="A2:C2"/>
+    <x:mergeCell ref="A1:D1"/>
+    <x:mergeCell ref="A2:D2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Support WB article imports for FF stocks
</commit_message>
<xml_diff>
--- a/public/ff-stock-import-template.xlsx
+++ b/public/ff-stock-import-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Остатки ФФ" sheetId="1" r:id="R7ae5f3bf5ec24dd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Остатки ФФ" sheetId="1" r:id="Ra844f7e1bf7b4355"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -527,7 +527,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="17" t="str">
-        <x:v>Артикул</x:v>
+        <x:v>Артикул WB</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
         <x:v>Партия</x:v>

</xml_diff>